<commit_message>
Increase header row heights to prevent logo overlapping row 4
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/elod_progresivos.xlsx
+++ b/output/elod_progresivos.xlsx
@@ -580,14 +580,14 @@
     <col width="5" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Federación Internacional de Léxico en Español (FILE)</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Elo Duplicada - Ranking Internacional</t>
@@ -599,6 +599,7 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="25" customHeight="1"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Center Row 2 subtitle+date across full width to avoid logo overlap
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/elod_progresivos.xlsx
+++ b/output/elod_progresivos.xlsx
@@ -590,12 +590,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Elo Duplicada - Ranking Internacional</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Actualizado al 8 de marzo de 2026</t>
+          <t>Elo Duplicada - Ranking Internacional  —  Actualizado al 8 de marzo de 2026</t>
         </is>
       </c>
     </row>
@@ -12674,10 +12669,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:BB1"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:BB2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix DeyaniraMarrera → DeyaniraMarrero (correct surname)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/elod_progresivos.xlsx
+++ b/output/elod_progresivos.xlsx
@@ -12197,12 +12197,12 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>MARRERA, Deyanira</t>
+          <t>MARRERO, Deyanira</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E237" s="9" t="n">

</xml_diff>